<commit_message>
add approx conf int calcs.
For app methods
</commit_message>
<xml_diff>
--- a/reductions/data-for-tables/app_meth_combined.xlsx
+++ b/reductions/data-for-tables/app_meth_combined.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aarhusuniversitet-my.sharepoint.com/personal/au583430_uni_au_dk/Documents/Documents/GitHub/GD-NH3/reductions/data-for-tables/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\au594831\GitHub_repos\GD-NH3\reductions\data-for-tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="215" documentId="8_{5E20B5B0-32C7-431D-8683-E50ABE62E15A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3F13213D-20C6-4891-98DF-201B622AECF9}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C308600A-8A19-438C-9516-D6EE91348B9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24225" yWindow="3885" windowWidth="21600" windowHeight="12645" activeTab="1" xr2:uid="{7C63DCD4-7913-4208-A171-6214FA8E3972}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{7C63DCD4-7913-4208-A171-6214FA8E3972}"/>
   </bookViews>
   <sheets>
     <sheet name="info" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="37">
   <si>
     <t>Trail hose</t>
   </si>
@@ -131,13 +131,34 @@
   </si>
   <si>
     <t>NA</t>
+  </si>
+  <si>
+    <t>rel. diff (%)</t>
+  </si>
+  <si>
+    <t>std. err.</t>
+  </si>
+  <si>
+    <t>lwr. lim.</t>
+  </si>
+  <si>
+    <t>upr. lim</t>
+  </si>
+  <si>
+    <t>n comb.</t>
+  </si>
+  <si>
+    <t>table val.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -171,6 +192,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -192,7 +219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -213,7 +240,8 @@
       <alignment horizontal="justify" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -549,39 +577,39 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D466B58A-D4CA-478A-9675-C91FBFEFB3AE}">
   <dimension ref="B3:B10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="43.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="43.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B4" s="2"/>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B5" s="6" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B6" s="6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B7" s="2"/>
     </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B8" s="2"/>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B9" s="2"/>
     </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B10" s="2"/>
     </row>
   </sheetData>
@@ -591,20 +619,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E141CA5-1FB4-4DAD-BBC1-66FB61386D09}">
-  <dimension ref="A1:N1048565"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:T1048565"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.28515625" customWidth="1"/>
-    <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" customWidth="1"/>
-    <col min="5" max="5" width="14.42578125" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" customWidth="1"/>
-    <col min="7" max="7" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.33203125" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.44140625" customWidth="1"/>
+    <col min="5" max="5" width="14.44140625" customWidth="1"/>
+    <col min="6" max="6" width="12.44140625" customWidth="1"/>
+    <col min="7" max="7" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.33203125" customWidth="1"/>
+    <col min="20" max="20" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" ht="30" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>12</v>
       </c>
@@ -615,10 +646,10 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
       <c r="C4" s="4"/>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
@@ -649,8 +680,26 @@
       <c r="M5" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N5" t="s">
+        <v>31</v>
+      </c>
+      <c r="O5" t="s">
+        <v>35</v>
+      </c>
+      <c r="P5" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>33</v>
+      </c>
+      <c r="R5" t="s">
+        <v>34</v>
+      </c>
+      <c r="T5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>1</v>
       </c>
@@ -682,8 +731,32 @@
         <f>(C6*B6+H6*J6)/(B6+J6)</f>
         <v>70.802730146315625</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N6" s="8">
+        <f>100*(H6-C6)/C6</f>
+        <v>-16.789079414737461</v>
+      </c>
+      <c r="O6" s="8">
+        <f>B6+J6</f>
+        <v>15</v>
+      </c>
+      <c r="P6" s="9">
+        <f>I6/SQRT(O6)</f>
+        <v>10.724248640396532</v>
+      </c>
+      <c r="Q6">
+        <f>M6-_xlfn.T.INV.2T(0.05, O6)*P6</f>
+        <v>47.944535255272413</v>
+      </c>
+      <c r="R6">
+        <f>MIN(M6+_xlfn.T.INV.2T(0.05, O6)*P6,100)</f>
+        <v>93.660925037358837</v>
+      </c>
+      <c r="T6" t="str">
+        <f>_xlfn.CONCAT(ROUND(M6,0), " [",ROUND(Q6,0), ", ", ROUND(R6,0), "]")</f>
+        <v>71 [48, 94]</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>2</v>
       </c>
@@ -715,8 +788,32 @@
         <f>(C7*B7+H7*J7)/(B7+J7)</f>
         <v>90.388469121858648</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N7" s="8">
+        <f t="shared" ref="N7:N9" si="0">100*(H7-C7)/C7</f>
+        <v>-6.7959402414714685</v>
+      </c>
+      <c r="O7" s="8">
+        <f t="shared" ref="O7:O10" si="1">B7+J7</f>
+        <v>7</v>
+      </c>
+      <c r="P7" s="9">
+        <f t="shared" ref="P7:P10" si="2">I7/SQRT(O7)</f>
+        <v>6.3314344184658893</v>
+      </c>
+      <c r="Q7">
+        <f t="shared" ref="Q7:Q10" si="3">M7-_xlfn.T.INV.2T(0.05, O7)*P7</f>
+        <v>75.417005748584941</v>
+      </c>
+      <c r="R7">
+        <f t="shared" ref="R7:R10" si="4">MIN(M7+_xlfn.T.INV.2T(0.05, O7)*P7,100)</f>
+        <v>100</v>
+      </c>
+      <c r="T7" t="str">
+        <f t="shared" ref="T7:T10" si="5">_xlfn.CONCAT(ROUND(M7,0), " [",ROUND(Q7,0), ", ", ROUND(R7,0), "]")</f>
+        <v>90 [75, 100]</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>3</v>
       </c>
@@ -748,8 +845,32 @@
         <f>(C8*B8+H8*J8)/(B8+J8)</f>
         <v>57.604258833907394</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N8" s="8">
+        <f>100*(H8-C8)/C8</f>
+        <v>-49.966727860098437</v>
+      </c>
+      <c r="O8" s="8">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="P8" s="9">
+        <f t="shared" si="2"/>
+        <v>17.48257378757188</v>
+      </c>
+      <c r="Q8">
+        <f t="shared" si="3"/>
+        <v>12.663872215403543</v>
+      </c>
+      <c r="R8">
+        <f t="shared" si="4"/>
+        <v>100</v>
+      </c>
+      <c r="T8" t="str">
+        <f t="shared" si="5"/>
+        <v>58 [13, 100]</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>0</v>
       </c>
@@ -781,182 +902,78 @@
         <f>(C9*B9+H9*J9)/(B9+J9)</f>
         <v>32.250860900784353</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N9" s="8">
+        <f t="shared" si="0"/>
+        <v>-36.812183236865984</v>
+      </c>
+      <c r="O9" s="8">
+        <f t="shared" si="1"/>
+        <v>17</v>
+      </c>
+      <c r="P9" s="9">
+        <f t="shared" si="2"/>
+        <v>13.969629162548634</v>
+      </c>
+      <c r="Q9">
+        <f t="shared" si="3"/>
+        <v>2.7775196770846513</v>
+      </c>
+      <c r="R9">
+        <f t="shared" si="4"/>
+        <v>61.724202124484052</v>
+      </c>
+      <c r="T9" t="str">
+        <f t="shared" si="5"/>
+        <v>32 [3, 62]</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A10" s="3"/>
-      <c r="G10" s="8" t="s">
+      <c r="G10" t="s">
         <v>25</v>
       </c>
-      <c r="H10" s="8">
+      <c r="H10">
         <v>43.744308969184402</v>
       </c>
-      <c r="I10" s="8">
+      <c r="I10">
         <v>22.843474281528799</v>
       </c>
-      <c r="J10" s="8">
+      <c r="J10">
         <v>6</v>
       </c>
-      <c r="K10" s="8"/>
-      <c r="L10" s="8"/>
-      <c r="M10" s="8">
+      <c r="M10">
         <f>H10</f>
         <v>43.744308969184402</v>
       </c>
       <c r="N10" s="8"/>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O10" s="8">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="P10" s="9">
+        <f t="shared" si="2"/>
+        <v>9.325809323689354</v>
+      </c>
+      <c r="Q10">
+        <f t="shared" si="3"/>
+        <v>20.924875613530666</v>
+      </c>
+      <c r="R10">
+        <f t="shared" si="4"/>
+        <v>66.563742324838131</v>
+      </c>
+      <c r="T10" t="str">
+        <f t="shared" si="5"/>
+        <v>44 [21, 67]</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A11" s="3"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8"/>
-      <c r="K11" s="8"/>
-      <c r="L11" s="8"/>
-      <c r="M11" s="8"/>
-      <c r="N11" s="8"/>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A12" s="3"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
-      <c r="K12" s="8"/>
-      <c r="L12" s="8"/>
-      <c r="M12" s="8"/>
-      <c r="N12" s="8"/>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
-      <c r="K13" s="8"/>
-      <c r="L13" s="8"/>
-      <c r="M13" s="8"/>
-      <c r="N13" s="8"/>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="G14" s="8"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="8"/>
-      <c r="J14" s="8"/>
-      <c r="K14" s="8"/>
-      <c r="L14" s="8"/>
-      <c r="M14" s="8"/>
-      <c r="N14" s="8"/>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="G15" s="8"/>
-      <c r="H15" s="8"/>
-      <c r="I15" s="8"/>
-      <c r="J15" s="8"/>
-      <c r="K15" s="8"/>
-      <c r="L15" s="8"/>
-      <c r="M15" s="8"/>
-      <c r="N15" s="8"/>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="8"/>
-      <c r="K16" s="8"/>
-      <c r="L16" s="8"/>
-      <c r="M16" s="8"/>
-      <c r="N16" s="8"/>
-    </row>
-    <row r="17" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="8"/>
-      <c r="K17" s="8"/>
-      <c r="L17" s="8"/>
-      <c r="M17" s="8"/>
-      <c r="N17" s="8"/>
-    </row>
-    <row r="18" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="8"/>
-      <c r="K18" s="8"/>
-      <c r="L18" s="8"/>
-      <c r="M18" s="8"/>
-      <c r="N18" s="8"/>
-    </row>
-    <row r="19" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
-      <c r="K19" s="8"/>
-      <c r="L19" s="8"/>
-      <c r="M19" s="8"/>
-      <c r="N19" s="8"/>
-    </row>
-    <row r="20" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
-      <c r="K20" s="8"/>
-      <c r="L20" s="8"/>
-      <c r="M20" s="8"/>
-      <c r="N20" s="8"/>
-    </row>
-    <row r="21" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
-      <c r="J21" s="8"/>
-      <c r="K21" s="8"/>
-      <c r="L21" s="8"/>
-      <c r="M21" s="8"/>
-      <c r="N21" s="8"/>
-    </row>
-    <row r="22" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G22" s="8"/>
-      <c r="H22" s="8"/>
-      <c r="I22" s="8"/>
-      <c r="J22" s="8"/>
-      <c r="K22" s="8"/>
-      <c r="L22" s="8"/>
-      <c r="M22" s="8"/>
-      <c r="N22" s="8"/>
-    </row>
-    <row r="23" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G23" s="8"/>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
-      <c r="J23" s="8"/>
-      <c r="K23" s="8"/>
-      <c r="L23" s="8"/>
-      <c r="M23" s="8"/>
-      <c r="N23" s="8"/>
-    </row>
-    <row r="24" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G24" s="8"/>
-      <c r="H24" s="8"/>
-      <c r="I24" s="8"/>
-      <c r="J24" s="8"/>
-      <c r="K24" s="8"/>
-      <c r="L24" s="8"/>
-      <c r="M24" s="8"/>
-      <c r="N24" s="8"/>
-    </row>
-    <row r="25" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G25" s="8"/>
-      <c r="H25" s="8"/>
-      <c r="I25" s="8"/>
-      <c r="J25" s="8"/>
-      <c r="K25" s="8"/>
-      <c r="L25" s="8"/>
-      <c r="M25" s="8"/>
-      <c r="N25" s="8"/>
-    </row>
-    <row r="1048565" spans="1:1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="1048565" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1048565" s="1"/>
     </row>
   </sheetData>
@@ -968,12 +985,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A7EE847-4537-48AE-B9AE-83B9CCAEBD54}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="37.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>13</v>
       </c>
@@ -987,7 +1004,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1004,7 +1021,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1021,7 +1038,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1038,7 +1055,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1055,7 +1072,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1072,7 +1089,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1089,7 +1106,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1106,7 +1123,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1123,7 +1140,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1140,7 +1157,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
unknown additional change to xlsx
</commit_message>
<xml_diff>
--- a/reductions/data-for-tables/app_meth_combined.xlsx
+++ b/reductions/data-for-tables/app_meth_combined.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\au594831\GitHub_repos\GD-NH3\reductions\data-for-tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C308600A-8A19-438C-9516-D6EE91348B9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D6DB4BE-D41C-4E29-B07A-67ED344E6109}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{7C63DCD4-7913-4208-A171-6214FA8E3972}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="38">
   <si>
     <t>Trail hose</t>
   </si>
@@ -149,6 +149,9 @@
   </si>
   <si>
     <t>table val.</t>
+  </si>
+  <si>
+    <t>t crit</t>
   </si>
 </sst>
 </file>
@@ -156,7 +159,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -241,7 +244,7 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -619,7 +622,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E141CA5-1FB4-4DAD-BBC1-66FB61386D09}">
-  <dimension ref="A1:T1048565"/>
+  <dimension ref="A1:U1048565"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.33203125" customWidth="1"/>
@@ -631,11 +634,11 @@
     <col min="7" max="7" width="26.88671875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="10.33203125" customWidth="1"/>
-    <col min="20" max="20" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="30" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" ht="30" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>12</v>
       </c>
@@ -646,10 +649,10 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="C4" s="4"/>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
@@ -690,16 +693,19 @@
         <v>32</v>
       </c>
       <c r="Q5" t="s">
+        <v>37</v>
+      </c>
+      <c r="R5" t="s">
         <v>33</v>
       </c>
-      <c r="R5" t="s">
+      <c r="S5" t="s">
         <v>34</v>
       </c>
-      <c r="T5" t="s">
+      <c r="U5" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>1</v>
       </c>
@@ -743,20 +749,24 @@
         <f>I6/SQRT(O6)</f>
         <v>10.724248640396532</v>
       </c>
-      <c r="Q6">
-        <f>M6-_xlfn.T.INV.2T(0.05, O6)*P6</f>
+      <c r="Q6" s="9">
+        <f>_xlfn.T.INV.2T(0.05, O6)</f>
+        <v>2.1314495455597742</v>
+      </c>
+      <c r="R6">
+        <f>M6-Q6*P6</f>
         <v>47.944535255272413</v>
       </c>
-      <c r="R6">
-        <f>MIN(M6+_xlfn.T.INV.2T(0.05, O6)*P6,100)</f>
+      <c r="S6">
+        <f>MIN(M6+Q6*P6,100)</f>
         <v>93.660925037358837</v>
       </c>
-      <c r="T6" t="str">
-        <f>_xlfn.CONCAT(ROUND(M6,0), " [",ROUND(Q6,0), ", ", ROUND(R6,0), "]")</f>
+      <c r="U6" t="str">
+        <f>_xlfn.CONCAT(ROUND(M6,0), " [",ROUND(R6,0), ", ", ROUND(S6,0), "]")</f>
         <v>71 [48, 94]</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>2</v>
       </c>
@@ -800,20 +810,24 @@
         <f t="shared" ref="P7:P10" si="2">I7/SQRT(O7)</f>
         <v>6.3314344184658893</v>
       </c>
-      <c r="Q7">
-        <f t="shared" ref="Q7:Q10" si="3">M7-_xlfn.T.INV.2T(0.05, O7)*P7</f>
+      <c r="Q7" s="9">
+        <f t="shared" ref="Q7:Q10" si="3">_xlfn.T.INV.2T(0.05, O7)</f>
+        <v>2.3646242515927849</v>
+      </c>
+      <c r="R7">
+        <f t="shared" ref="R7:R10" si="4">M7-Q7*P7</f>
         <v>75.417005748584941</v>
       </c>
-      <c r="R7">
-        <f t="shared" ref="R7:R10" si="4">MIN(M7+_xlfn.T.INV.2T(0.05, O7)*P7,100)</f>
+      <c r="S7">
+        <f t="shared" ref="S7:S10" si="5">MIN(M7+Q7*P7,100)</f>
         <v>100</v>
       </c>
-      <c r="T7" t="str">
-        <f t="shared" ref="T7:T10" si="5">_xlfn.CONCAT(ROUND(M7,0), " [",ROUND(Q7,0), ", ", ROUND(R7,0), "]")</f>
+      <c r="U7" t="str">
+        <f t="shared" ref="U7:U10" si="6">_xlfn.CONCAT(ROUND(M7,0), " [",ROUND(R7,0), ", ", ROUND(S7,0), "]")</f>
         <v>90 [75, 100]</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>3</v>
       </c>
@@ -857,20 +871,24 @@
         <f t="shared" si="2"/>
         <v>17.48257378757188</v>
       </c>
-      <c r="Q8">
+      <c r="Q8" s="9">
         <f t="shared" si="3"/>
-        <v>12.663872215403543</v>
+        <v>2.570581835636315</v>
       </c>
       <c r="R8">
         <f t="shared" si="4"/>
+        <v>12.663872215403543</v>
+      </c>
+      <c r="S8">
+        <f t="shared" si="5"/>
         <v>100</v>
       </c>
-      <c r="T8" t="str">
-        <f t="shared" si="5"/>
+      <c r="U8" t="str">
+        <f t="shared" si="6"/>
         <v>58 [13, 100]</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>0</v>
       </c>
@@ -914,20 +932,24 @@
         <f t="shared" si="2"/>
         <v>13.969629162548634</v>
       </c>
-      <c r="Q9">
+      <c r="Q9" s="9">
         <f t="shared" si="3"/>
-        <v>2.7775196770846513</v>
+        <v>2.109815577833317</v>
       </c>
       <c r="R9">
         <f t="shared" si="4"/>
+        <v>2.7775196770846513</v>
+      </c>
+      <c r="S9">
+        <f t="shared" si="5"/>
         <v>61.724202124484052</v>
       </c>
-      <c r="T9" t="str">
-        <f t="shared" si="5"/>
+      <c r="U9" t="str">
+        <f t="shared" si="6"/>
         <v>32 [3, 62]</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10" s="3"/>
       <c r="G10" t="s">
         <v>25</v>
@@ -954,23 +976,27 @@
         <f t="shared" si="2"/>
         <v>9.325809323689354</v>
       </c>
-      <c r="Q10">
+      <c r="Q10" s="9">
         <f t="shared" si="3"/>
-        <v>20.924875613530666</v>
+        <v>2.4469118511449697</v>
       </c>
       <c r="R10">
         <f t="shared" si="4"/>
+        <v>20.924875613530666</v>
+      </c>
+      <c r="S10">
+        <f t="shared" si="5"/>
         <v>66.563742324838131</v>
       </c>
-      <c r="T10" t="str">
-        <f t="shared" si="5"/>
+      <c r="U10" t="str">
+        <f t="shared" si="6"/>
         <v>44 [21, 67]</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11" s="3"/>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A12" s="3"/>
     </row>
     <row r="1048565" spans="1:1" x14ac:dyDescent="0.3">

</xml_diff>